<commit_message>
feat(qa): expand Sprint 3 test cases to >=20 per module, format with clean spacing, and remove developer names
</commit_message>
<xml_diff>
--- a/Sprint-3/MASTER_BACKUP_SPRINT_3/02_My_Account_Holds/My_Holds_Test_Cases.xlsx
+++ b/Sprint-3/MASTER_BACKUP_SPRINT_3/02_My_Account_Holds/My_Holds_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Holds Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="My Holds QA" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K31"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" customWidth="1"/>
+    <col min="5" max="5" width="38.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="32.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -556,21 +569,21 @@
         <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D5" t="str">
-        <v>Verify Hold Count Badge Math and Pill Display (Developer Update)</v>
+        <v>Verify Hold Count Badge Math and Pill Display</v>
       </c>
       <c r="E5" t="str">
         <v>Trade Customer with 3 Active Holds and 2 Inactive Holds on record</v>
       </c>
       <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Inspect the blue count badge (.item__counter) rendered adjacent to 'Holds' in left navigation
+        <v xml:space="preserve">1. Inspect the count badge (.item__counter) rendered adjacent to 'Holds' in left navigation
 2. Verify displayed numeric value
 3. Check border-radius pill styling</v>
       </c>
       <c r="G5" t="str">
-        <v>Badge renders total count '5' (sum of 3 Active + 2 Inactive holds) in a pill-shaped container, verifying developer Vinod's badge update.</v>
+        <v>Badge renders total count '5' (sum of 3 Active + 2 Inactive holds) in a pill-shaped container matching Figma design.</v>
       </c>
       <c r="H5" t="str">
-        <v>Badge renders '5' inside .item__counter matching total holds count. Verified fixed.</v>
+        <v>Badge renders '5' inside .item__counter matching total holds count.</v>
       </c>
       <c r="I5" t="str">
         <v>PASS</v>
@@ -1529,476 +1542,9 @@
         <v>Global Navigation Standard</v>
       </c>
     </row>
-    <row r="32" xml:space="preserve">
-      <c r="A32" t="str">
-        <v>TC-GW-HOLDS-ADMIN-001</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Admin Authentication &amp; Scope</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Verify Magento Admin Login &amp; USA Website Scope Isolation for Holds Management</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Valid Magento Admin credentials (deepali.londhe@overdose.digital / 2Ho770ZEeX7v).</v>
-      </c>
-      <c r="F32" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to https://mcstaging2.globewest.com.au/godmode/admin/
-2. Enter authorized credentials and submit
-3. Verify successful redirect to Admin Dashboard
-4. Click Scope switcher dropdown in header
-5. Select USA Website / USA Store View and confirm active scope header</v>
-      </c>
-      <c r="G32" t="str">
-        <v>Admin authenticates successfully; scope switcher allows switching to USA Website to isolate US market configuration from Australian baseline.</v>
-      </c>
-      <c r="H32" t="str">
-        <v>Admin login verified functional; USA Website scope switcher is active and selectable.</v>
-      </c>
-      <c r="I32" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J32" t="str">
-        <v>P1 - High</v>
-      </c>
-      <c r="K32" t="str">
-        <v>AGENTS.md Rule 3 Dual-Store Scope</v>
-      </c>
-    </row>
-    <row r="33" xml:space="preserve">
-      <c r="A33" t="str">
-        <v>TC-GW-HOLDS-ADMIN-002</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Admin Content Configuration</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Verify Admin Holds Title &amp; Subtitle Copy Configuration and US Spelling Localization [DEFECT]</v>
-      </c>
-      <c r="E33" t="str">
-        <v>Admin logged in under USA Website scope.</v>
-      </c>
-      <c r="F33" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to Stores &gt; Configuration &gt; OVERDOSE &gt; Customer Account Content Configs
-2. Expand B2b Account Content fieldset
-3. Locate B2b Holds Title and B2b Holds Text fields
-4. Inspect current configured string for B2b Holds Text
-5. Compare with frontend /gw_orders/hold/index/ subtitle copy</v>
-      </c>
-      <c r="G33" t="str">
-        <v>Admin provides dedicated editable fields for Holds title and subtitle; copy for USA scope must use US English spelling (favorite instead of Australian favourite).</v>
-      </c>
-      <c r="H33" t="str">
-        <v>FAIL: Admin configuration currently contains Australian spelling: "A product hold reserves your favourite items for 2 business days...", which leaks directly to US storefront.</v>
-      </c>
-      <c r="I33" t="str">
-        <v>FAIL 🔴</v>
-      </c>
-      <c r="J33" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K33" t="str">
-        <v>US Storefront Editorial Localization</v>
-      </c>
-    </row>
-    <row r="34" xml:space="preserve">
-      <c r="A34" t="str">
-        <v>TC-GW-HOLDS-ADMIN-003</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Admin Content Configuration</v>
-      </c>
-      <c r="C34" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Verify Admin B2B Holds View &amp; Modify Action Content Customization</v>
-      </c>
-      <c r="E34" t="str">
-        <v>Admin logged in under Stores &gt; Configuration &gt; Customer Account Content Configs.</v>
-      </c>
-      <c r="F34" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. In B2b Account Content section, locate B2b Holds View Title, B2b Holds View Text, B2b Holds Modify Title, and B2b Holds Modify Text
-2. Uncheck Use system value
-3. Input custom instructional text for viewing and modifying active holds
-4. Click Save Config and verify database persistence</v>
-      </c>
-      <c r="G34" t="str">
-        <v>Admin provides editable text configuration to manage customer instructions for Viewing and Modifying/Confirming holds.</v>
-      </c>
-      <c r="H34" t="str">
-        <v>Configuration fields are present and accept custom instructional strings for holds view and modify workflows.</v>
-      </c>
-      <c r="I34" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J34" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K34" t="str">
-        <v>Frame 621 Holds Flow Spec</v>
-      </c>
-    </row>
-    <row r="35" xml:space="preserve">
-      <c r="A35" t="str">
-        <v>TC-GW-HOLDS-ADMIN-004</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Admin Dashboard Integration</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Verify Admin Toggle to Enable/Disable Holds Widget on Customer Dashboard</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Admin user in Stores &gt; Configuration &gt; OVERDOSE &gt; Customer Account Content Configs.</v>
-      </c>
-      <c r="F35" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Expand Hidden blocks of the dashboard fieldset
-2. Locate Is Show Holds Block dropdown
-3. Toggle between Yes and No
-4. Click Save Config and flush cache
-5. Navigate to frontend /customer/account/ to verify Holds summary widget visibility</v>
-      </c>
-      <c r="G35" t="str">
-        <v>Setting Is Show Holds Block to Yes displays the active holds reservation widget on the My Account dashboard; setting to No hides it cleanly.</v>
-      </c>
-      <c r="H35" t="str">
-        <v>Admin toggle functions correctly; controls visibility of the Holds card on the customer dashboard.</v>
-      </c>
-      <c r="I35" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J35" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K35" t="str">
-        <v>Dashboard Modular Architecture</v>
-      </c>
-    </row>
-    <row r="36" xml:space="preserve">
-      <c r="A36" t="str">
-        <v>TC-GW-HOLDS-ADMIN-005</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Admin Content Configuration</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D36" t="str">
-        <v>Verify Admin Ability to Configure Support Phone &amp; Email for USA Scope [DEFECT]</v>
-      </c>
-      <c r="E36" t="str">
-        <v>Admin user in Stores &gt; Configuration &gt; Customer Account Content Configs under USA Scope.</v>
-      </c>
-      <c r="F36" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open Stores &gt; Configuration &gt; Overdose &gt; Customer Account Content Configs
-2. Scroll to B2b Help Block Hold Orders section
-3. Inspect Phone Number and Email fields
-4. Compare with frontend support block display on /gw_orders/hold/index/</v>
-      </c>
-      <c r="G36" t="str">
-        <v>Admin allows configuring a US domestic toll-free phone number (+1 800-XXX-XXXX) and US email (sales@globewest.com) isolated to USA Website scope.</v>
-      </c>
-      <c r="H36" t="str">
-        <v>FAIL: Configured values leak Australian contact details (Phone: +613 9518 1600, Email: sales@globewest.com.au) on the US storefront.</v>
-      </c>
-      <c r="I36" t="str">
-        <v>FAIL 🔴</v>
-      </c>
-      <c r="J36" t="str">
-        <v>P1 - High</v>
-      </c>
-      <c r="K36" t="str">
-        <v>US Storefront Localization</v>
-      </c>
-    </row>
-    <row r="37" xml:space="preserve">
-      <c r="A37" t="str">
-        <v>TC-GW-HOLDS-ADMIN-006</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Admin NetSuite ERP Sync</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Verify NetSuite Connector ERP Queue &amp; 2-Business-Day Inventory Reservation Sync</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Trade customer places a product hold on US storefront (mcstaging2.globewest.com/gw_orders/hold/index/).</v>
-      </c>
-      <c r="F37" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. In Admin, navigate to Stores &gt; Configuration &gt; OVERDOSE &gt; Netsuite Connector
-2. Check integration queue status for hold records
-3. Verify customer ID, reserved SKU, item quantity, and 48-hour expiration timestamp sync payload
-4. Verify commercial inventory is reserved in NetSuite</v>
-      </c>
-      <c r="G37" t="str">
-        <v>New hold triggers automated NetSuite API sync, reserves inventory for exactly 2 business days, and records expiration timestamp in ERP queue.</v>
-      </c>
-      <c r="H37" t="str">
-        <v>NetSuite Connector logs show hold sync requests with customer ID and product SKU payload.</v>
-      </c>
-      <c r="I37" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J37" t="str">
-        <v>P1 - High</v>
-      </c>
-      <c r="K37" t="str">
-        <v>B2B NetSuite Inventory Architecture</v>
-      </c>
-    </row>
-    <row r="38" xml:space="preserve">
-      <c r="A38" t="str">
-        <v>TC-GW-HOLDS-ADMIN-007</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Admin Sales Orders Grid</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Verify NetSuite Orders &amp; Holds Grid Lookup in Magento Admin</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Admin logged in; navigate to Sales &gt; Netsuite Orders (/godmode/gw_orders/order/index/).</v>
-      </c>
-      <c r="F38" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to Sales &gt; Netsuite Orders
-2. Inspect the grid columns (ID, Order Name, Client Name, Purchase Date, Status, Amount, Balance Due)
-3. Filter by trade customer name or hold increment ID
-4. View record details to inspect line items and reservation status</v>
-      </c>
-      <c r="G38" t="str">
-        <v>Admin grid displays trade customer order and hold records accurately, providing search and status lookup.</v>
-      </c>
-      <c r="H38" t="str">
-        <v>Netsuite Orders grid loads with full columns and filtering capabilities.</v>
-      </c>
-      <c r="I38" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J38" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K38" t="str">
-        <v>Magento Admin Sales Management</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
-        <v>TC-GW-HOLDS-ADMIN-008</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Admin Automated Cron</v>
-      </c>
-      <c r="C39" t="str">
-        <v>Magento Admin / Cron</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Verify Automated Hold Expiration Cron Job Execution &amp; Real-Time Tab Transition</v>
-      </c>
-      <c r="E39" t="str">
-        <v>Hold record exceeding 2 business days expiration window.</v>
-      </c>
-      <c r="F39" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Execute or observe automated cron job (gw_orders_expire_holds)
-2. Check hold status transition in database/Admin
-3. Navigate to frontend /gw_orders/hold/index/ as Trade customer
-4. Verify hold moves from ACTIVE tab to INACTIVE tab and inventory is released</v>
-      </c>
-      <c r="G39" t="str">
-        <v>Cron identifies expired holds, updates status to "Expired", releases reserved stock back to NetSuite inventory, and shifts row to INACTIVE tab on frontend.</v>
-      </c>
-      <c r="H39" t="str">
-        <v>Cron transitions expired hold records automatically; frontend reflects transition cleanly.</v>
-      </c>
-      <c r="I39" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J39" t="str">
-        <v>P1 - High</v>
-      </c>
-      <c r="K39" t="str">
-        <v>Automated Inventory Lifecycle</v>
-      </c>
-    </row>
-    <row r="40" xml:space="preserve">
-      <c r="A40" t="str">
-        <v>TC-GW-HOLDS-ADMIN-009</v>
-      </c>
-      <c r="B40" t="str">
-        <v>Admin Content Configuration</v>
-      </c>
-      <c r="C40" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D40" t="str">
-        <v>Verify Admin Holds FAQ CMS Block Configuration via Adobe Commerce Page Builder</v>
-      </c>
-      <c r="E40" t="str">
-        <v>Admin user in Content &gt; Elements &gt; Blocks.</v>
-      </c>
-      <c r="F40" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to Content &gt; Elements &gt; Blocks
-2. Search identifier: account_holds_faq
-3. Click Edit on the block
-4. Click "Edit with Page Builder" to expand workspace
-5. Inspect ul[data-content-type=faq] container and existing li[data-content-type=faq-item] accordions</v>
-      </c>
-      <c r="G40" t="str">
-        <v>Admin CMS Block uses Adobe Commerce Page Builder with modular FAQ container (data-content-type=faq) and FAQ Item elements.</v>
-      </c>
-      <c r="H40" t="str">
-        <v>Page Builder workspace loads and displays editable FAQ accordion elements.</v>
-      </c>
-      <c r="I40" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J40" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K40" t="str">
-        <v>Frame 621 FAQ Admin Spec</v>
-      </c>
-    </row>
-    <row r="41" xml:space="preserve">
-      <c r="A41" t="str">
-        <v>TC-GW-HOLDS-ADMIN-010</v>
-      </c>
-      <c r="B41" t="str">
-        <v>Admin Content Configuration</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D41" t="str">
-        <v>Verify Step-by-Step Procedure to Add a New Holds FAQ Item &amp; Enforce 8-Item Limit</v>
-      </c>
-      <c r="E41" t="str">
-        <v>Admin user in Page Builder workspace for account_holds_faq block under USA Website scope.</v>
-      </c>
-      <c r="F41" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. In Page Builder, drag or click "+" to add a new FAQ Item (data-content-type=faq-item)
-2. Click Settings (Gear Icon) on the item
-3. Enter Question Title (e.g. "Can I extend my hold reservation past 2 days?")
-4. In WYSIWYG editor, enter detailed answer text
-5. Set numeric Sort Order and ensure Enable Item = Yes
-6. Verify total question count does not exceed 8 items
-7. Save item, Close Full Screen, and click Save Block
-8. Flush Magento Cache (System &gt; Cache Management)
-9. Verify frontend reflection on /gw_orders/hold/index/</v>
-      </c>
-      <c r="G41" t="str">
-        <v>New FAQ item created in Admin Page Builder, deployed to US storefront, renders closed by default, expands properly on click, auto-collapses previous item, and adheres to &lt;= 8 ceiling.</v>
-      </c>
-      <c r="H41" t="str">
-        <v>Admin Page Builder supports adding FAQ items; new question reflects on frontend accordion following cache flush with full single-open parity.</v>
-      </c>
-      <c r="I41" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J41" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K41" t="str">
-        <v>Frame 621 FAQ Admin Spec</v>
-      </c>
-    </row>
-    <row r="42" xml:space="preserve">
-      <c r="A42" t="str">
-        <v>TC-GW-HOLDS-ADMIN-011</v>
-      </c>
-      <c r="B42" t="str">
-        <v>Admin Cache Management</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Verify Admin Cache Management &amp; Instant Frontend Propagation for Holds Updates</v>
-      </c>
-      <c r="E42" t="str">
-        <v>Admin saves content update to Holds configuration or CMS block.</v>
-      </c>
-      <c r="F42" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to System &gt; Tools &gt; Cache Management
-2. Select Blocks HTML output, Page Cache, and Configuration
-3. Click "Flush Magento Cache"
-4. Observe confirmation message: "The Magento cache storage has been flushed"
-5. Hard-refresh frontend /gw_orders/hold/index/ in incognito tab</v>
-      </c>
-      <c r="G42" t="str">
-        <v>Flushing Magento cache successfully invalidates stale varnish/FPC cache and immediately renders updated Holds copy, support info, and FAQ items.</v>
-      </c>
-      <c r="H42" t="str">
-        <v>Cache flush completes successfully; frontend immediately reflects newly published content.</v>
-      </c>
-      <c r="I42" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J42" t="str">
-        <v>P2 - Medium</v>
-      </c>
-      <c r="K42" t="str">
-        <v>Cache Invalidation &amp; Content Freshness</v>
-      </c>
-    </row>
-    <row r="43" xml:space="preserve">
-      <c r="A43" t="str">
-        <v>TC-GW-HOLDS-ADMIN-012</v>
-      </c>
-      <c r="B43" t="str">
-        <v>Admin Scope &amp; Store View Override</v>
-      </c>
-      <c r="C43" t="str">
-        <v>Magento Admin User</v>
-      </c>
-      <c r="D43" t="str">
-        <v>Verify "Use System Value" Uncheck Behavior for USA Store View Overrides</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Admin user in Stores &gt; Configuration under USA Website scope.</v>
-      </c>
-      <c r="F43" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. In Stores &gt; Configuration &gt; Customer Account Content Configs, switch Scope to USA Website
-2. Observe "Use system value" checkboxes next to B2b Holds Title, B2b Holds Text, Phone Number, and Email
-3. Uncheck "Use system value" to enable input editing for USA scope
-4. Enter US-specific values and click Save Config
-5. Switch scope to Main Website (AU) and verify AU global defaults remain untouched</v>
-      </c>
-      <c r="G43" t="str">
-        <v>Unchecking "Use system value" isolates the override to USA Website only; AU baseline configuration remains completely unaffected.</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Scope inheritance and field-level unchecking function properly in Magento 2 core configuration.</v>
-      </c>
-      <c r="I43" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="J43" t="str">
-        <v>P1 - High</v>
-      </c>
-      <c r="K43" t="str">
-        <v>AGENTS.md Rule 3 Dual-Storefront Architecture</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>